<commit_message>
feat(qa): three runners (web, Android, iOS) over one scenario source
- UiDriver contract + Playwright/Appium adapters
- screens rewritten as platform-neutral page objects
- smoke/e2e scenarios defined once, executed by all runners
- tests/web (Playwright) + tests/native (WDIO/Mocha) harnesses
- runners/{playwright,wdio.shared,wdio.android,wdio.ios}.conf.js
- CI matrix: web, Android emulator, iOS simulator
- docs/PLATFORMS.md: matrix, emulator setup, verified status

web: 30/30 passing (5 smoke, 15 e2e, 10 regression)
</commit_message>
<xml_diff>
--- a/docs/HostelHub_TestCases.xlsx
+++ b/docs/HostelHub_TestCases.xlsx
@@ -21,7 +21,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-10-25 18:44:48 UTC</t>
+    <t>2026-10-25 19:19:49 UTC</t>
   </si>
   <si>
     <t>Web under test</t>
@@ -180,7 +180,7 @@
     <t>n/a</t>
   </si>
   <si>
-    <t>tests/smoke/critical-paths.spec.js › SMK-01 API health endpoint responds</t>
+    <t>tests/web/smoke.spec.js › SMK-01 API health endpoint responds</t>
   </si>
   <si>
     <t>SMK-02</t>
@@ -199,7 +199,7 @@
     <t>"Welcome back", Username and Password fields, Log in button are present</t>
   </si>
   <si>
-    <t>tests/smoke/critical-paths.spec.js › SMK-02 app loads and shows the login screen</t>
+    <t>tests/web/smoke.spec.js › SMK-02 app loads and shows the login screen</t>
   </si>
   <si>
     <t>SMK-03</t>
@@ -221,7 +221,7 @@
     <t>owner seeded per run</t>
   </si>
   <si>
-    <t>tests/smoke/critical-paths.spec.js › SMK-03 owner signs in and sees the dashboard</t>
+    <t>tests/web/smoke.spec.js › SMK-03 owner signs in and sees the dashboard</t>
   </si>
   <si>
     <t>SMK-04</t>
@@ -244,7 +244,7 @@
     <t>Every tab renders without the router error page; Home returns to the dashboard</t>
   </si>
   <si>
-    <t>tests/smoke/critical-paths.spec.js › SMK-04 owner tabs are all reachable</t>
+    <t>tests/web/smoke.spec.js › SMK-04 owner tabs are all reachable</t>
   </si>
   <si>
     <t>SMK-05</t>
@@ -266,7 +266,7 @@
     <t>resident seeded</t>
   </si>
   <si>
-    <t>tests/smoke/critical-paths.spec.js › SMK-05 seeded resident is listed on the inmates tab</t>
+    <t>tests/web/smoke.spec.js › SMK-05 seeded resident is listed on the inmates tab</t>
   </si>
   <si>
     <t>E2E-AUTH-01</t>
@@ -289,7 +289,7 @@
     <t>owner seeded</t>
   </si>
   <si>
-    <t>tests/e2e/auth.spec.js › E2E-AUTH-01 owner signs in with valid credentials</t>
+    <t>tests/web/auth.spec.js › E2E-AUTH-01 owner signs in with valid credentials</t>
   </si>
   <si>
     <t>E2E-AUTH-02</t>
@@ -311,7 +311,7 @@
     <t>WrongPass!1</t>
   </si>
   <si>
-    <t>tests/e2e/auth.spec.js › E2E-AUTH-02 invalid password keeps the user on the login screen</t>
+    <t>tests/web/auth.spec.js › E2E-AUTH-02 invalid password keeps the user on the login screen</t>
   </si>
   <si>
     <t>E2E-AUTH-03</t>
@@ -332,7 +332,7 @@
     <t>Create-account screen is displayed</t>
   </si>
   <si>
-    <t>tests/e2e/auth.spec.js › E2E-AUTH-03 sign-up screen opens from login</t>
+    <t>tests/web/auth.spec.js › E2E-AUTH-03 sign-up screen opens from login</t>
   </si>
   <si>
     <t>E2E-AUTH-04</t>
@@ -347,7 +347,7 @@
     <t>Password reset screen is displayed</t>
   </si>
   <si>
-    <t>tests/e2e/auth.spec.js › E2E-AUTH-04 forgot-password screen opens from login</t>
+    <t>tests/web/auth.spec.js › E2E-AUTH-04 forgot-password screen opens from login</t>
   </si>
   <si>
     <t>E2E-AUTH-05</t>
@@ -365,7 +365,7 @@
     <t>Router redirects to /login and the login screen renders</t>
   </si>
   <si>
-    <t>tests/e2e/auth.spec.js › E2E-AUTH-05 protected route redirects to login when signed out</t>
+    <t>tests/web/auth.spec.js › E2E-AUTH-05 protected route redirects to login when signed out</t>
   </si>
   <si>
     <t>E2E-AUTH-06</t>
@@ -382,7 +382,7 @@
     <t>Session cleared and the login screen is shown</t>
   </si>
   <si>
-    <t>tests/e2e/auth.spec.js › E2E-AUTH-06 owner can sign out</t>
+    <t>tests/web/auth.spec.js › E2E-AUTH-06 owner can sign out</t>
   </si>
   <si>
     <t>REG-SES-01</t>
@@ -397,7 +397,7 @@
     <t>User stays on /home and the dashboard re-renders</t>
   </si>
   <si>
-    <t>tests/regression/session.spec.js › REG-SES-01 session survives a page reload</t>
+    <t>tests/web/regression.spec.jssession.spec.js › REG-SES-01 session survives a page reload</t>
   </si>
   <si>
     <t>REG-SES-02</t>
@@ -412,7 +412,7 @@
     <t>No navigation; route stays /login</t>
   </si>
   <si>
-    <t>tests/regression/session.spec.js › REG-SES-02 empty credentials do not navigate</t>
+    <t>tests/web/regression.spec.jssession.spec.js › REG-SES-02 empty credentials do not navigate</t>
   </si>
   <si>
     <t>REG-SES-03</t>
@@ -427,7 +427,7 @@
     <t>Each route redirects to /login</t>
   </si>
   <si>
-    <t>tests/regression/session.spec.js › REG-SES-03 every protected route redirects to login when signed out</t>
+    <t>tests/web/regression.spec.jssession.spec.js › REG-SES-03 every protected route redirects to login when signed out</t>
   </si>
   <si>
     <t>REG-SES-04</t>
@@ -443,7 +443,7 @@
     <t>App returns to the login screen, no session restored</t>
   </si>
   <si>
-    <t>tests/regression/session.spec.js › REG-SES-04 logout clears the session</t>
+    <t>tests/web/regression.spec.jssession.spec.js › REG-SES-04 logout clears the session</t>
   </si>
   <si>
     <t>E2E-ONB-01</t>
@@ -464,7 +464,7 @@
     <t>fresh owner</t>
   </si>
   <si>
-    <t>tests/e2e/onboarding.spec.js › E2E-ONB-01 new owner sees the setup prompt</t>
+    <t>tests/web/onboarding.spec.js › E2E-ONB-01 new owner sees the setup prompt</t>
   </si>
   <si>
     <t>E2E-ONB-02</t>
@@ -482,7 +482,7 @@
     <t>Wizard renders its first step without an error page</t>
   </si>
   <si>
-    <t>tests/e2e/onboarding.spec.js › E2E-ONB-02 setup wizard opens from the prompt</t>
+    <t>tests/web/onboarding.spec.js › E2E-ONB-02 setup wizard opens from the prompt</t>
   </si>
   <si>
     <t>E2E-ONB-03</t>
@@ -504,7 +504,7 @@
     <t>property + room seeded</t>
   </si>
   <si>
-    <t>tests/e2e/onboarding.spec.js › E2E-ONB-03 property + rooms appear on the dashboard and inmates tab</t>
+    <t>tests/web/onboarding.spec.js › E2E-ONB-03 property + rooms appear on the dashboard and inmates tab</t>
   </si>
   <si>
     <t>MNL-ONB-01</t>
@@ -546,7 +546,7 @@
     <t>Property name, Rooms section and the resident are listed</t>
   </si>
   <si>
-    <t>tests/e2e/inmates.spec.js › E2E-INM-01 inmates tab shows the property, rooms and residents</t>
+    <t>tests/web/inmates.spec.js › E2E-INM-01 inmates tab shows the property, rooms and residents</t>
   </si>
   <si>
     <t>E2E-INM-02</t>
@@ -570,7 +570,7 @@
     <t>bed 2, rent 7000, due day 10</t>
   </si>
   <si>
-    <t>tests/e2e/inmates.spec.js › E2E-INM-02 owner adds a resident through the form</t>
+    <t>tests/web/inmates.spec.js › E2E-INM-02 owner adds a resident through the form</t>
   </si>
   <si>
     <t>E2E-INM-03</t>
@@ -589,7 +589,7 @@
     <t>bed 3</t>
   </si>
   <si>
-    <t>tests/e2e/inmates.spec.js › E2E-INM-03 the resident created in the UI exists in the API</t>
+    <t>tests/web/inmates.spec.js › E2E-INM-03 the resident created in the UI exists in the API</t>
   </si>
   <si>
     <t>REG-OCC-01</t>
@@ -611,7 +611,7 @@
     <t>capacity 3</t>
   </si>
   <si>
-    <t>tests/regression/occupancy.spec.js › REG-OCC-01 a room cannot exceed its capacity</t>
+    <t>tests/web/regression.spec.jsoccupancy.spec.js › REG-OCC-01 a room cannot exceed its capacity</t>
   </si>
   <si>
     <t>REG-OCC-02</t>
@@ -632,7 +632,7 @@
     <t>bed 1</t>
   </si>
   <si>
-    <t>tests/regression/occupancy.spec.js › REG-OCC-02 a bed cannot be assigned twice</t>
+    <t>tests/web/regression.spec.jsoccupancy.spec.js › REG-OCC-02 a bed cannot be assigned twice</t>
   </si>
   <si>
     <t>REG-OCC-03</t>
@@ -650,7 +650,7 @@
     <t>bed 99</t>
   </si>
   <si>
-    <t>tests/regression/occupancy.spec.js › REG-OCC-03 bed number outside 1..capacity is rejected</t>
+    <t>tests/web/regression.spec.jsoccupancy.spec.js › REG-OCC-03 bed number outside 1..capacity is rejected</t>
   </si>
   <si>
     <t>REG-OCC-04</t>
@@ -669,7 +669,7 @@
     <t>Listed with the same room_no, bed_no and rent_amount</t>
   </si>
   <si>
-    <t>tests/regression/occupancy.spec.js › REG-OCC-04 an API-created resident appears with room and bed</t>
+    <t>tests/web/regression.spec.jsoccupancy.spec.js › REG-OCC-04 an API-created resident appears with room and bed</t>
   </si>
   <si>
     <t>MNL-INM-02</t>
@@ -746,7 +746,7 @@
     <t>meal=dinner</t>
   </si>
   <si>
-    <t>tests/e2e/polls.spec.js › E2E-POLL-01 polls tab renders an active poll</t>
+    <t>tests/web/polls.spec.js › E2E-POLL-01 polls tab renders an active poll</t>
   </si>
   <si>
     <t>E2E-POLL-02</t>
@@ -764,7 +764,7 @@
     <t>options === ["Yes","No"], recurring is true/false</t>
   </si>
   <si>
-    <t>tests/e2e/polls.spec.js › E2E-POLL-02 API returns poll options as an array and recurring as boolean</t>
+    <t>tests/web/polls.spec.js › E2E-POLL-02 API returns poll options as an array and recurring as boolean</t>
   </si>
   <si>
     <t>E2E-POLL-03</t>
@@ -783,7 +783,7 @@
     <t>Every returned poll belongs to the requested property</t>
   </si>
   <si>
-    <t>tests/e2e/polls.spec.js › E2E-POLL-03 poll creation is scoped to the property</t>
+    <t>tests/web/polls.spec.js › E2E-POLL-03 poll creation is scoped to the property</t>
   </si>
   <si>
     <t>MNL-POLL-01</t>
@@ -816,7 +816,7 @@
     <t>Complaints list renders with an empty state or entries</t>
   </si>
   <si>
-    <t>tests/e2e/ops.spec.js › E2E-OPS-01 complaints screen renders</t>
+    <t>tests/web/ops.spec.js › E2E-OPS-01 complaints screen renders</t>
   </si>
   <si>
     <t>E2E-OPS-02</t>
@@ -831,7 +831,7 @@
     <t>Documents screen plus "Add hostel document"</t>
   </si>
   <si>
-    <t>tests/e2e/ops.spec.js › E2E-OPS-02 documents screen renders with its upload action</t>
+    <t>tests/web/ops.spec.js › E2E-OPS-02 documents screen renders with its upload action</t>
   </si>
   <si>
     <t>E2E-OPS-03</t>
@@ -846,7 +846,7 @@
     <t>P&amp;L header, income, expenses and net are displayed</t>
   </si>
   <si>
-    <t>tests/e2e/ops.spec.js › E2E-OPS-03 expenses screen shows the P&amp;L summary</t>
+    <t>tests/web/ops.spec.js › E2E-OPS-03 expenses screen shows the P&amp;L summary</t>
   </si>
   <si>
     <t>E2E-OPS-04</t>
@@ -861,7 +861,7 @@
     <t>Each screen renders its heading with no router error page</t>
   </si>
   <si>
-    <t>tests/e2e/ops.spec.js › E2E-OPS-04 visitors, deposits, ratings and SOS render</t>
+    <t>tests/web/ops.spec.js › E2E-OPS-04 visitors, deposits, ratings and SOS render</t>
   </si>
   <si>
     <t>E2E-OPS-05</t>
@@ -870,7 +870,7 @@
     <t>Settings, bills and chat render</t>
   </si>
   <si>
-    <t>tests/e2e/ops.spec.js › E2E-OPS-05 settings, bills and chat render</t>
+    <t>tests/web/ops.spec.js › E2E-OPS-05 settings, bills and chat render</t>
   </si>
   <si>
     <t>E2E-OPS-06</t>
@@ -890,7 +890,7 @@
     <t>Electricity 1200</t>
   </si>
   <si>
-    <t>tests/e2e/ops.spec.js › E2E-OPS-06 adding an expense reaches the P&amp;L endpoint</t>
+    <t>tests/web/ops.spec.js › E2E-OPS-06 adding an expense reaches the P&amp;L endpoint</t>
   </si>
   <si>
     <t>MNL-OPS-01</t>
@@ -946,7 +946,7 @@
     <t>health is {status:"ok"}; pricing.global has monthly, yearly, extra_property numbers</t>
   </si>
   <si>
-    <t>tests/regression/api.contract.spec.js › REG-API-01</t>
+    <t>tests/web/regression.spec.jsapi.contract.spec.js › REG-API-01</t>
   </si>
   <si>
     <t>REG-API-02</t>
@@ -968,7 +968,7 @@
     <t>new owner</t>
   </si>
   <si>
-    <t>tests/regression/api.contract.spec.js › REG-API-02</t>
+    <t>tests/web/regression.spec.jsapi.contract.spec.js › REG-API-02</t>
   </si>
   <si>
     <t>REG-API-03</t>
@@ -986,7 +986,7 @@
     <t>401 and the response body does not contain the password</t>
   </si>
   <si>
-    <t>tests/regression/api.contract.spec.js › REG-API-03</t>
+    <t>tests/web/regression.spec.jsapi.contract.spec.js › REG-API-03</t>
   </si>
   <si>
     <t>REG-API-04</t>
@@ -1007,7 +1007,7 @@
     <t>existing username</t>
   </si>
   <si>
-    <t>tests/regression/api.contract.spec.js › REG-API-04</t>
+    <t>tests/web/regression.spec.jsapi.contract.spec.js › REG-API-04</t>
   </si>
   <si>
     <t>REG-API-05</t>
@@ -1025,7 +1025,7 @@
     <t>true/false (a 0 breaks the Flutter models)</t>
   </si>
   <si>
-    <t>tests/regression/api.contract.spec.js › REG-API-05</t>
+    <t>tests/web/regression.spec.jsapi.contract.spec.js › REG-API-05</t>
   </si>
   <si>
     <t>REG-API-06</t>
@@ -1047,7 +1047,7 @@
     <t>tenant A / B</t>
   </si>
   <si>
-    <t>tests/regression/api.contract.spec.js › REG-API-06</t>
+    <t>tests/web/regression.spec.jsapi.contract.spec.js › REG-API-06</t>
   </si>
   <si>
     <t>MNL-API-01</t>
@@ -1133,7 +1133,7 @@
     <t>Login screen with Username and Password fields</t>
   </si>
   <si>
-    <t>tests/mobile/auth.mobile.test.js › MOB-AUTH-01</t>
+    <t>tests/native/auth.mobile.test.js › MOB-AUTH-01</t>
   </si>
   <si>
     <t>MOB-AUTH-02</t>
@@ -1152,7 +1152,7 @@
     <t>Dashboard renders with the owner tabs</t>
   </si>
   <si>
-    <t>tests/mobile/auth.mobile.test.js › MOB-AUTH-02</t>
+    <t>tests/native/auth.mobile.test.js › MOB-AUTH-02</t>
   </si>
   <si>
     <t>MOB-NAV-01</t>
@@ -1171,7 +1171,7 @@
     <t>Residents listed, dashboard restored</t>
   </si>
   <si>
-    <t>tests/mobile/navigation.mobile.test.js › MOB-NAV-01</t>
+    <t>tests/native/navigation.mobile.test.js › MOB-NAV-01</t>
   </si>
   <si>
     <t>External issue ID</t>
@@ -1214,7 +1214,7 @@
 *Expected result:*
 200 with {"status":"ok"}
 *Test data:* n/a
-*Automated by:* tests/smoke/critical-paths.spec.js › SMK-01 API health endpoint responds</t>
+*Automated by:* tests/web/smoke.spec.js › SMK-01 API health endpoint responds</t>
   </si>
   <si>
     <t>SMK-02 — App loads and shows the login screen</t>
@@ -1234,7 +1234,7 @@
 *Expected result:*
 "Welcome back", Username and Password fields, Log in button are present
 *Test data:* n/a
-*Automated by:* tests/smoke/critical-paths.spec.js › SMK-02 app loads and shows the login screen</t>
+*Automated by:* tests/web/smoke.spec.js › SMK-02 app loads and shows the login screen</t>
   </si>
   <si>
     <t>SMK-03 — Owner signs in and sees the dashboard</t>
@@ -1254,7 +1254,7 @@
 *Expected result:*
 Dashboard shows the property name and the KPI cards (Inmates, Occupancy, Rooms, Pending dues)
 *Test data:* owner seeded per run
-*Automated by:* tests/smoke/critical-paths.spec.js › SMK-03 owner signs in and sees the dashboard</t>
+*Automated by:* tests/web/smoke.spec.js › SMK-03 owner signs in and sees the dashboard</t>
   </si>
   <si>
     <t>SMK-04 — All owner tabs are reachable</t>
@@ -1275,7 +1275,7 @@
 *Expected result:*
 Every tab renders without the router error page; Home returns to the dashboard
 *Test data:* n/a
-*Automated by:* tests/smoke/critical-paths.spec.js › SMK-04 owner tabs are all reachable</t>
+*Automated by:* tests/web/smoke.spec.js › SMK-04 owner tabs are all reachable</t>
   </si>
   <si>
     <t>SMK-05 — Seeded resident is listed on the inmates tab</t>
@@ -1295,7 +1295,7 @@
 *Expected result:*
 The resident name is listed
 *Test data:* resident seeded
-*Automated by:* tests/smoke/critical-paths.spec.js › SMK-05 seeded resident is listed on the inmates tab</t>
+*Automated by:* tests/web/smoke.spec.js › SMK-05 seeded resident is listed on the inmates tab</t>
   </si>
   <si>
     <t>E2E-AUTH-01 — Owner signs in with valid credentials</t>
@@ -1319,7 +1319,7 @@
 *Expected result:*
 User lands on /home and the dashboard renders for their property
 *Test data:* owner seeded
-*Automated by:* tests/e2e/auth.spec.js › E2E-AUTH-01 owner signs in with valid credentials</t>
+*Automated by:* tests/web/auth.spec.js › E2E-AUTH-01 owner signs in with valid credentials</t>
   </si>
   <si>
     <t>E2E-AUTH-02 — Invalid password keeps the user on the login screen</t>
@@ -1339,7 +1339,7 @@
 *Expected result:*
 Error message shown, route stays /login
 *Test data:* WrongPass!1
-*Automated by:* tests/e2e/auth.spec.js › E2E-AUTH-02 invalid password keeps the user on the login screen</t>
+*Automated by:* tests/web/auth.spec.js › E2E-AUTH-02 invalid password keeps the user on the login screen</t>
   </si>
   <si>
     <t>E2E-AUTH-03 — Sign-up screen opens from login</t>
@@ -1361,7 +1361,7 @@
 *Expected result:*
 Create-account screen is displayed
 *Test data:* n/a
-*Automated by:* tests/e2e/auth.spec.js › E2E-AUTH-03 sign-up screen opens from login</t>
+*Automated by:* tests/web/auth.spec.js › E2E-AUTH-03 sign-up screen opens from login</t>
   </si>
   <si>
     <t>E2E-AUTH-04 — Forgot-password screen opens from login</t>
@@ -1380,7 +1380,7 @@
 *Expected result:*
 Password reset screen is displayed
 *Test data:* n/a
-*Automated by:* tests/e2e/auth.spec.js › E2E-AUTH-04 forgot-password screen opens from login</t>
+*Automated by:* tests/web/auth.spec.js › E2E-AUTH-04 forgot-password screen opens from login</t>
   </si>
   <si>
     <t>E2E-AUTH-05 — Protected route redirects to login when signed out</t>
@@ -1399,7 +1399,7 @@
 *Expected result:*
 Router redirects to /login and the login screen renders
 *Test data:* n/a
-*Automated by:* tests/e2e/auth.spec.js › E2E-AUTH-05 protected route redirects to login when signed out</t>
+*Automated by:* tests/web/auth.spec.js › E2E-AUTH-05 protected route redirects to login when signed out</t>
   </si>
   <si>
     <t>E2E-AUTH-06 — Owner can sign out</t>
@@ -1420,7 +1420,7 @@
 *Expected result:*
 Session cleared and the login screen is shown
 *Test data:* n/a
-*Automated by:* tests/e2e/auth.spec.js › E2E-AUTH-06 owner can sign out</t>
+*Automated by:* tests/web/auth.spec.js › E2E-AUTH-06 owner can sign out</t>
   </si>
   <si>
     <t>REG-SES-01 — Session survives a page reload</t>
@@ -1442,7 +1442,7 @@
 *Expected result:*
 User stays on /home and the dashboard re-renders
 *Test data:* n/a
-*Automated by:* tests/regression/session.spec.js › REG-SES-01 session survives a page reload</t>
+*Automated by:* tests/web/regression.spec.jssession.spec.js › REG-SES-01 session survives a page reload</t>
   </si>
   <si>
     <t>REG-SES-02 — Empty credentials do not navigate</t>
@@ -1464,7 +1464,7 @@
 *Expected result:*
 No navigation; route stays /login
 *Test data:* n/a
-*Automated by:* tests/regression/session.spec.js › REG-SES-02 empty credentials do not navigate</t>
+*Automated by:* tests/web/regression.spec.jssession.spec.js › REG-SES-02 empty credentials do not navigate</t>
   </si>
   <si>
     <t>REG-SES-03 — Every protected route redirects when signed out</t>
@@ -1483,7 +1483,7 @@
 *Expected result:*
 Each route redirects to /login
 *Test data:* n/a
-*Automated by:* tests/regression/session.spec.js › REG-SES-03 every protected route redirects to login when signed out</t>
+*Automated by:* tests/web/regression.spec.jssession.spec.js › REG-SES-03 every protected route redirects to login when signed out</t>
   </si>
   <si>
     <t>REG-SES-04 — Logout clears the persisted session</t>
@@ -1503,7 +1503,7 @@
 *Expected result:*
 App returns to the login screen, no session restored
 *Test data:* n/a
-*Automated by:* tests/regression/session.spec.js › REG-SES-04 logout clears the session</t>
+*Automated by:* tests/web/regression.spec.jssession.spec.js › REG-SES-04 logout clears the session</t>
   </si>
   <si>
     <t>E2E-ONB-01 — New owner sees the setup prompt</t>
@@ -1522,7 +1522,7 @@
 *Expected result:*
 "Set up your hostel" prompt with a Get started button
 *Test data:* fresh owner
-*Automated by:* tests/e2e/onboarding.spec.js › E2E-ONB-01 new owner sees the setup prompt</t>
+*Automated by:* tests/web/onboarding.spec.js › E2E-ONB-01 new owner sees the setup prompt</t>
   </si>
   <si>
     <t>E2E-ONB-02 — Setup wizard opens from the prompt</t>
@@ -1541,7 +1541,7 @@
 *Expected result:*
 Wizard renders its first step without an error page
 *Test data:* n/a
-*Automated by:* tests/e2e/onboarding.spec.js › E2E-ONB-02 setup wizard opens from the prompt</t>
+*Automated by:* tests/web/onboarding.spec.js › E2E-ONB-02 setup wizard opens from the prompt</t>
   </si>
   <si>
     <t>E2E-ONB-03 — Property and rooms appear on dashboard and inmates tab</t>
@@ -1561,7 +1561,7 @@
 *Expected result:*
 Property name on both screens; rooms section present
 *Test data:* property + room seeded
-*Automated by:* tests/e2e/onboarding.spec.js › E2E-ONB-03 property + rooms appear on the dashboard and inmates tab</t>
+*Automated by:* tests/web/onboarding.spec.js › E2E-ONB-03 property + rooms appear on the dashboard and inmates tab</t>
   </si>
   <si>
     <t>MNL-ONB-01 — Complete the setup wizard end to end</t>
@@ -1605,7 +1605,7 @@
 *Expected result:*
 Property name, Rooms section and the resident are listed
 *Test data:* resident seeded
-*Automated by:* tests/e2e/inmates.spec.js › E2E-INM-01 inmates tab shows the property, rooms and residents</t>
+*Automated by:* tests/web/inmates.spec.js › E2E-INM-01 inmates tab shows the property, rooms and residents</t>
   </si>
   <si>
     <t>E2E-INM-02 — Owner adds a resident through the form</t>
@@ -1627,7 +1627,7 @@
 *Expected result:*
 Resident created, credentials shown, resident listed afterwards
 *Test data:* bed 2, rent 7000, due day 10
-*Automated by:* tests/e2e/inmates.spec.js › E2E-INM-02 owner adds a resident through the form</t>
+*Automated by:* tests/web/inmates.spec.js › E2E-INM-02 owner adds a resident through the form</t>
   </si>
   <si>
     <t>E2E-INM-03 — Resident created in the UI exists in the API</t>
@@ -1647,7 +1647,7 @@
 *Expected result:*
 The API returns the resident with the same room and bed
 *Test data:* bed 3
-*Automated by:* tests/e2e/inmates.spec.js › E2E-INM-03 the resident created in the UI exists in the API</t>
+*Automated by:* tests/web/inmates.spec.js › E2E-INM-03 the resident created in the UI exists in the API</t>
   </si>
   <si>
     <t>REG-OCC-01 — Room capacity cannot be exceeded</t>
@@ -1667,7 +1667,7 @@
 *Expected result:*
 API rejects with a "room is full" error
 *Test data:* capacity 3
-*Automated by:* tests/regression/occupancy.spec.js › REG-OCC-01 a room cannot exceed its capacity</t>
+*Automated by:* tests/web/regression.spec.jsoccupancy.spec.js › REG-OCC-01 a room cannot exceed its capacity</t>
   </si>
   <si>
     <t>REG-OCC-02 — A bed cannot be assigned twice</t>
@@ -1686,7 +1686,7 @@
 *Expected result:*
 API rejects with "bed already taken"
 *Test data:* bed 1
-*Automated by:* tests/regression/occupancy.spec.js › REG-OCC-02 a bed cannot be assigned twice</t>
+*Automated by:* tests/web/regression.spec.jsoccupancy.spec.js › REG-OCC-02 a bed cannot be assigned twice</t>
   </si>
   <si>
     <t>REG-OCC-03 — Bed number outside the room range is rejected</t>
@@ -1705,7 +1705,7 @@
 *Expected result:*
 API rejects with "bed out of range"
 *Test data:* bed 99
-*Automated by:* tests/regression/occupancy.spec.js › REG-OCC-03 bed number outside 1..capacity is rejected</t>
+*Automated by:* tests/web/regression.spec.jsoccupancy.spec.js › REG-OCC-03 bed number outside 1..capacity is rejected</t>
   </si>
   <si>
     <t>REG-OCC-04 — API-created resident exposes room and bed</t>
@@ -1725,7 +1725,7 @@
 *Expected result:*
 Listed with the same room_no, bed_no and rent_amount
 *Test data:* n/a
-*Automated by:* tests/regression/occupancy.spec.js › REG-OCC-04 an API-created resident appears with room and bed</t>
+*Automated by:* tests/web/regression.spec.jsoccupancy.spec.js › REG-OCC-04 an API-created resident appears with room and bed</t>
   </si>
   <si>
     <t>MNL-INM-02 — Regenerate resident credentials</t>
@@ -1812,7 +1812,7 @@
 *Expected result:*
 Poll is listed with its meal and options
 *Test data:* meal=dinner
-*Automated by:* tests/e2e/polls.spec.js › E2E-POLL-01 polls tab renders an active poll</t>
+*Automated by:* tests/web/polls.spec.js › E2E-POLL-01 polls tab renders an active poll</t>
   </si>
   <si>
     <t>E2E-POLL-02 — Poll options are an array and recurring is a boolean</t>
@@ -1831,7 +1831,7 @@
 *Expected result:*
 options === ["Yes","No"], recurring is true/false
 *Test data:* n/a
-*Automated by:* tests/e2e/polls.spec.js › E2E-POLL-02 API returns poll options as an array and recurring as boolean</t>
+*Automated by:* tests/web/polls.spec.js › E2E-POLL-02 API returns poll options as an array and recurring as boolean</t>
   </si>
   <si>
     <t>E2E-POLL-03 — Polls are scoped to their property</t>
@@ -1851,7 +1851,7 @@
 *Expected result:*
 Every returned poll belongs to the requested property
 *Test data:* n/a
-*Automated by:* tests/e2e/polls.spec.js › E2E-POLL-03 poll creation is scoped to the property</t>
+*Automated by:* tests/web/polls.spec.js › E2E-POLL-03 poll creation is scoped to the property</t>
   </si>
   <si>
     <t>MNL-POLL-01 — Resident answers a poll and the owner sees the headcount</t>
@@ -1892,7 +1892,7 @@
 *Expected result:*
 Complaints list renders with an empty state or entries
 *Test data:* n/a
-*Automated by:* tests/e2e/ops.spec.js › E2E-OPS-01 complaints screen renders</t>
+*Automated by:* tests/web/ops.spec.js › E2E-OPS-01 complaints screen renders</t>
   </si>
   <si>
     <t>E2E-OPS-02 — Documents screen renders with its upload action</t>
@@ -1911,7 +1911,7 @@
 *Expected result:*
 Documents screen plus "Add hostel document"
 *Test data:* n/a
-*Automated by:* tests/e2e/ops.spec.js › E2E-OPS-02 documents screen renders with its upload action</t>
+*Automated by:* tests/web/ops.spec.js › E2E-OPS-02 documents screen renders with its upload action</t>
   </si>
   <si>
     <t>E2E-OPS-03 — Expenses screen shows the P&amp;L summary</t>
@@ -1930,7 +1930,7 @@
 *Expected result:*
 P&amp;L header, income, expenses and net are displayed
 *Test data:* n/a
-*Automated by:* tests/e2e/ops.spec.js › E2E-OPS-03 expenses screen shows the P&amp;L summary</t>
+*Automated by:* tests/web/ops.spec.js › E2E-OPS-03 expenses screen shows the P&amp;L summary</t>
   </si>
   <si>
     <t>E2E-OPS-04 — Visitors, deposits, ratings and SOS render</t>
@@ -1949,7 +1949,7 @@
 *Expected result:*
 Each screen renders its heading with no router error page
 *Test data:* n/a
-*Automated by:* tests/e2e/ops.spec.js › E2E-OPS-04 visitors, deposits, ratings and SOS render</t>
+*Automated by:* tests/web/ops.spec.js › E2E-OPS-04 visitors, deposits, ratings and SOS render</t>
   </si>
   <si>
     <t>E2E-OPS-05 — Settings, bills and chat render</t>
@@ -1968,7 +1968,7 @@
 *Expected result:*
 Each screen renders its heading with no router error page
 *Test data:* n/a
-*Automated by:* tests/e2e/ops.spec.js › E2E-OPS-05 settings, bills and chat render</t>
+*Automated by:* tests/web/ops.spec.js › E2E-OPS-05 settings, bills and chat render</t>
   </si>
   <si>
     <t>E2E-OPS-06 — Adding an expense reaches the P&amp;L endpoint</t>
@@ -1989,7 +1989,7 @@
 *Expected result:*
 GET /pnl returns income, expense and net as numbers
 *Test data:* Electricity 1200
-*Automated by:* tests/e2e/ops.spec.js › E2E-OPS-06 adding an expense reaches the P&amp;L endpoint</t>
+*Automated by:* tests/web/ops.spec.js › E2E-OPS-06 adding an expense reaches the P&amp;L endpoint</t>
   </si>
   <si>
     <t>MNL-OPS-01 — Raise and resolve a complaint</t>
@@ -2051,7 +2051,7 @@
 *Expected result:*
 health is {status:"ok"}; pricing.global has monthly, yearly, extra_property numbers
 *Test data:* n/a
-*Automated by:* tests/regression/api.contract.spec.js › REG-API-01</t>
+*Automated by:* tests/web/regression.spec.jsapi.contract.spec.js › REG-API-01</t>
   </si>
   <si>
     <t>REG-API-02 — Register and login issue a signed JWT</t>
@@ -2071,7 +2071,7 @@
 *Expected result:*
 Three-part JWT; user payload never contains the password
 *Test data:* new owner
-*Automated by:* tests/regression/api.contract.spec.js › REG-API-02</t>
+*Automated by:* tests/web/regression.spec.jsapi.contract.spec.js › REG-API-02</t>
   </si>
   <si>
     <t>REG-API-03 — Wrong password is 401 without echoing the password</t>
@@ -2090,7 +2090,7 @@
 *Expected result:*
 401 and the response body does not contain the password
 *Test data:* WrongPass!1
-*Automated by:* tests/regression/api.contract.spec.js › REG-API-03</t>
+*Automated by:* tests/web/regression.spec.jsapi.contract.spec.js › REG-API-03</t>
   </si>
   <si>
     <t>REG-API-04 — Duplicate username is rejected</t>
@@ -2109,7 +2109,7 @@
 *Expected result:*
 400 or 409 with a clear message
 *Test data:* existing username
-*Automated by:* tests/regression/api.contract.spec.js › REG-API-04</t>
+*Automated by:* tests/web/regression.spec.jsapi.contract.spec.js › REG-API-04</t>
   </si>
   <si>
     <t>REG-API-05 — Boolean fields are real JSON booleans</t>
@@ -2128,7 +2128,7 @@
 *Expected result:*
 true/false (a 0 breaks the Flutter models)
 *Test data:* n/a
-*Automated by:* tests/regression/api.contract.spec.js › REG-API-05</t>
+*Automated by:* tests/web/regression.spec.jsapi.contract.spec.js › REG-API-05</t>
   </si>
   <si>
     <t>REG-API-06 — Tenants are isolated</t>
@@ -2148,7 +2148,7 @@
 *Expected result:*
 Each owner sees only their own property
 *Test data:* tenant A / B
-*Automated by:* tests/regression/api.contract.spec.js › REG-API-06</t>
+*Automated by:* tests/web/regression.spec.jsapi.contract.spec.js › REG-API-06</t>
   </si>
   <si>
     <t>MNL-API-01 — Worker secrets are configured</t>
@@ -2245,7 +2245,7 @@
 *Expected result:*
 Login screen with Username and Password fields
 *Test data:* n/a
-*Automated by:* tests/mobile/auth.mobile.test.js › MOB-AUTH-01</t>
+*Automated by:* tests/native/auth.mobile.test.js › MOB-AUTH-01</t>
   </si>
   <si>
     <t>MOB-AUTH-02 — Native app signs in with valid credentials</t>
@@ -2265,7 +2265,7 @@
 *Expected result:*
 Dashboard renders with the owner tabs
 *Test data:* owner seeded
-*Automated by:* tests/mobile/auth.mobile.test.js › MOB-AUTH-02</t>
+*Automated by:* tests/native/auth.mobile.test.js › MOB-AUTH-02</t>
   </si>
   <si>
     <t>MOB-NAV-01 — Native shell navigation works</t>
@@ -2285,7 +2285,7 @@
 *Expected result:*
 Residents listed, dashboard restored
 *Test data:* n/a
-*Automated by:* tests/mobile/navigation.mobile.test.js › MOB-NAV-01</t>
+*Automated by:* tests/native/navigation.mobile.test.js › MOB-NAV-01</t>
   </si>
 </sst>
 </file>

</xml_diff>